<commit_message>
qL and GW DO
</commit_message>
<xml_diff>
--- a/04_Output/rC_k600.xlsx
+++ b/04_Output/rC_k600.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samanthahowley\Desktop\Howley_Bradford_Streams\04_Output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howley_Bradford_Streams\Howley_Bradford_Streams\04_Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32BC8FE-C517-463B-AF04-3B578AC745CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{087B4428-3DB4-427A-BC09-98D1B60EB199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2220" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="13" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -70,6 +70,9 @@
     <t>k600_dh</t>
   </si>
   <si>
+    <t>KO2_1d</t>
+  </si>
+  <si>
     <t>KCO2_1d</t>
   </si>
   <si>
@@ -77,6 +80,12 @@
   </si>
   <si>
     <t>log_K600</t>
+  </si>
+  <si>
+    <t>sd</t>
+  </si>
+  <si>
+    <t>mean</t>
   </si>
   <si>
     <t>13</t>
@@ -105,12 +114,6 @@
   <si>
     <t>9</t>
   </si>
-  <si>
-    <t>mean</t>
-  </si>
-  <si>
-    <t>sd_k600</t>
-  </si>
 </sst>
 </file>
 
@@ -131,6 +134,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -452,10 +456,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N8"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O8"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,18 +497,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45231.643750000003</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2">
         <v>861.60841666666704</v>
@@ -516,7 +523,7 @@
         <v>9.6741420654558305E-2</v>
       </c>
       <c r="F2">
-        <v>11.645584669675101</v>
+        <v>11.9120522108645</v>
       </c>
       <c r="G2">
         <v>68.241833333333304</v>
@@ -528,29 +535,30 @@
         <v>2.3846125037819001E-2</v>
       </c>
       <c r="J2">
+        <v>-6.8042146345373098</v>
+      </c>
+      <c r="K2">
         <v>2.3294976165444799E-2</v>
       </c>
-      <c r="K2">
-        <v>2.4549271098625498</v>
-      </c>
       <c r="L2">
+        <v>2.47755067841983</v>
+      </c>
+      <c r="M2">
         <v>-3.7361335470566699</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45279.638888888898</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>682.46505000000002</v>
@@ -562,7 +570,7 @@
         <v>0.535585069806503</v>
       </c>
       <c r="F3">
-        <v>170.37625534230901</v>
+        <v>168.71047104642</v>
       </c>
       <c r="G3">
         <v>58.136791666666703</v>
@@ -574,29 +582,30 @@
         <v>4.16356543733956E-2</v>
       </c>
       <c r="J3">
+        <v>-1.7610548631285201</v>
+      </c>
+      <c r="K3">
         <v>3.3927945946732298E-2</v>
       </c>
-      <c r="K3">
-        <v>5.1380092581028904</v>
-      </c>
       <c r="L3">
+        <v>5.1281840566619898</v>
+      </c>
+      <c r="M3">
         <v>-3.1787984025115201</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M8" si="0">AVERAGE(I:I)</f>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N8" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45331.546296296299</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C4">
         <v>841.73281919999999</v>
@@ -608,7 +617,7 @@
         <v>0.173458550098919</v>
       </c>
       <c r="F4">
-        <v>25.528660174141699</v>
+        <v>25.9714864991385</v>
       </c>
       <c r="G4">
         <v>58.711833333333303</v>
@@ -616,27 +625,34 @@
       <c r="H4">
         <v>5.4401628671565296</v>
       </c>
+      <c r="I4">
+        <v>6.6050205004409301</v>
+      </c>
+      <c r="J4">
+        <v>872.72864896527597</v>
+      </c>
       <c r="K4">
-        <v>3.2398017494274298</v>
+        <v>5.4401628671565296</v>
       </c>
       <c r="L4">
+        <v>3.2569992631254499</v>
+      </c>
+      <c r="M4">
         <v>1.88783004174554</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45442.611111111102</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>749.64344000000006</v>
@@ -648,7 +664,7 @@
         <v>2.1803076333425399E-2</v>
       </c>
       <c r="F5">
-        <v>0.80426230095528795</v>
+        <v>0.85851602582766595</v>
       </c>
       <c r="G5">
         <v>73.386250000000004</v>
@@ -660,29 +676,30 @@
         <v>6.7770495933372303E-3</v>
       </c>
       <c r="J5">
+        <v>-9.4331831408977092</v>
+      </c>
+      <c r="K5">
         <v>7.2230120683586304E-3</v>
       </c>
-      <c r="K5">
-        <v>-0.217829818040225</v>
-      </c>
       <c r="L5">
+        <v>-0.15254993157636201</v>
+      </c>
+      <c r="M5">
         <v>-4.9942134349654204</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45569.592476851903</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6">
         <v>410.82921599999997</v>
@@ -694,7 +711,7 @@
         <v>7.2829882932493206E-2</v>
       </c>
       <c r="F6">
-        <v>5.9255578069466397</v>
+        <v>6.1548729066271699</v>
       </c>
       <c r="G6">
         <v>75.485124999999996</v>
@@ -706,29 +723,30 @@
         <v>2.47946706179097E-2</v>
       </c>
       <c r="J6">
+        <v>-10.729558156220699</v>
+      </c>
+      <c r="K6">
         <v>2.7360058733056799E-2</v>
       </c>
-      <c r="K6">
-        <v>1.7792748272222101</v>
-      </c>
       <c r="L6">
+        <v>1.81724411062179</v>
+      </c>
+      <c r="M6">
         <v>-3.6971265433434399</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45590.559143518498</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <v>380.73329999999999</v>
@@ -740,7 +758,7 @@
         <v>9.2027430068846006E-2</v>
       </c>
       <c r="F7">
-        <v>8.7927060696889594</v>
+        <v>9.0815785426951301</v>
       </c>
       <c r="G7">
         <v>68.770458333333295</v>
@@ -752,29 +770,30 @@
         <v>3.3803954304686301E-2</v>
       </c>
       <c r="J7">
+        <v>-10.242869195642401</v>
+      </c>
+      <c r="K7">
         <v>3.33313008490599E-2</v>
       </c>
-      <c r="K7">
-        <v>2.17392252207617</v>
-      </c>
       <c r="L7">
+        <v>2.2062480258177799</v>
+      </c>
+      <c r="M7">
         <v>-3.3871774920731998</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>1.1669123048760234E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45639.626736111102</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>350.53264000000001</v>
@@ -786,7 +805,7 @@
         <v>5.6819055456292601E-2</v>
       </c>
       <c r="F8">
-        <v>3.9102083694124099</v>
+        <v>4.0853145075861104</v>
       </c>
       <c r="G8">
         <v>56.352833333333301</v>
@@ -794,22 +813,26 @@
       <c r="H8">
         <v>-0.18731814069170799</v>
       </c>
+      <c r="I8">
+        <v>0.237662875388165</v>
+      </c>
       <c r="J8">
+        <v>-91.374797378565205</v>
+      </c>
+      <c r="K8">
         <v>0.18731814069170799</v>
       </c>
-      <c r="K8">
-        <v>1.36359066398716</v>
-      </c>
       <c r="L8">
+        <v>1.4073987161894801</v>
+      </c>
+      <c r="M8">
         <v>-1.4369020994466399</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>2.6171490785429567E-2</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>1.1669123048760234E-2</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -820,10 +843,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -861,18 +884,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45279.458796296298</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>743.79520000000002</v>
@@ -884,7 +910,7 @@
         <v>0.50826006985347305</v>
       </c>
       <c r="F2">
-        <v>697.91479401277002</v>
+        <v>705.23843021665402</v>
       </c>
       <c r="G2">
         <v>57.950125</v>
@@ -896,29 +922,30 @@
         <v>0.173934288769413</v>
       </c>
       <c r="J2">
+        <v>-7.7241163873473102</v>
+      </c>
+      <c r="K2">
         <v>0.14126099627199201</v>
       </c>
-      <c r="K2">
-        <v>6.54809702369608</v>
-      </c>
       <c r="L2">
+        <v>6.5585359445247899</v>
+      </c>
+      <c r="M2">
         <v>-1.7490777018461099</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45296.476041666698</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3">
         <v>638.45846666666705</v>
@@ -930,7 +957,7 @@
         <v>0.19585224806813301</v>
       </c>
       <c r="F3">
-        <v>24.3034926825508</v>
+        <v>24.587734986814599</v>
       </c>
       <c r="G3">
         <v>53.767708333333303</v>
@@ -942,29 +969,30 @@
         <v>2.5524128899415702E-2</v>
       </c>
       <c r="J3">
+        <v>-2.6988247333370401</v>
+      </c>
+      <c r="K3">
         <v>1.9154349794311701E-2</v>
       </c>
-      <c r="K3">
-        <v>3.1906200718102902</v>
-      </c>
       <c r="L3">
+        <v>3.2022477408353298</v>
+      </c>
+      <c r="M3">
         <v>-3.6681310428627998</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M11" si="0">AVERAGE(I:I)</f>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N11" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45484.508796296301</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C4">
         <v>792.39509999999996</v>
@@ -976,7 +1004,7 @@
         <v>0.21609790544256399</v>
       </c>
       <c r="F4">
-        <v>34.413560705227098</v>
+        <v>34.811732781454197</v>
       </c>
       <c r="G4">
         <v>76.441249999999997</v>
@@ -988,29 +1016,30 @@
         <v>0.33304642862635703</v>
       </c>
       <c r="J4">
+        <v>-49.402717452382703</v>
+      </c>
+      <c r="K4">
         <v>0.37328004715152302</v>
       </c>
-      <c r="K4">
-        <v>3.5384506932476598</v>
-      </c>
       <c r="L4">
+        <v>3.5499544788508799</v>
+      </c>
+      <c r="M4">
         <v>-1.0994733734161199</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45502.467245370397</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C5">
         <v>801.76949999999999</v>
@@ -1022,7 +1051,7 @@
         <v>0.29201786247728301</v>
       </c>
       <c r="F5">
-        <v>99.192565071371106</v>
+        <v>100.302711713524</v>
       </c>
       <c r="G5">
         <v>76.383166666666696</v>
@@ -1030,30 +1059,34 @@
       <c r="H5">
         <v>1.40185787623314</v>
       </c>
+      <c r="I5">
+        <v>1.2518618359821001</v>
+      </c>
       <c r="J5">
+        <v>137.28645747561899</v>
+      </c>
+      <c r="K5">
         <v>1.40185787623314</v>
       </c>
-      <c r="K5">
-        <v>4.5970630626047102</v>
-      </c>
       <c r="L5">
+        <v>4.6081927306295896</v>
+      </c>
+      <c r="M5">
         <v>0.22463191194150001</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45569.420833333301</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>693.87467000000004</v>
@@ -1065,7 +1098,7 @@
         <v>0.22996315545078599</v>
       </c>
       <c r="F6">
-        <v>42.788239065963701</v>
+        <v>43.279994270392898</v>
       </c>
       <c r="G6">
         <v>76.3036666666667</v>
@@ -1073,30 +1106,34 @@
       <c r="H6">
         <v>-2.7299788409758401</v>
       </c>
+      <c r="I6">
+        <v>2.44145804581688</v>
+      </c>
       <c r="J6">
+        <v>-339.451968582402</v>
+      </c>
+      <c r="K6">
         <v>2.7299788409758401</v>
       </c>
-      <c r="K6">
-        <v>3.7562632766481401</v>
-      </c>
       <c r="L6">
+        <v>3.76769050215358</v>
+      </c>
+      <c r="M6">
         <v>0.89259542059838703</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45590.410069444399</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>546.66366000000005</v>
@@ -1108,7 +1145,7 @@
         <v>0.14324969531057899</v>
       </c>
       <c r="F7">
-        <v>8.1262160020957896</v>
+        <v>8.2244229946684495</v>
       </c>
       <c r="G7">
         <v>69.349500000000006</v>
@@ -1120,29 +1157,30 @@
         <v>0.90949515581084905</v>
       </c>
       <c r="J7">
+        <v>178.956846560911</v>
+      </c>
+      <c r="K7">
         <v>0.90568158280436795</v>
       </c>
-      <c r="K7">
-        <v>2.0950953788139999</v>
-      </c>
       <c r="L7">
+        <v>2.1071081415667301</v>
+      </c>
+      <c r="M7">
         <v>-9.4865607249415299E-2</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45639.483333333301</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C8">
         <v>660.91974000000005</v>
@@ -1154,7 +1192,7 @@
         <v>8.0274044883753906E-2</v>
       </c>
       <c r="F8">
-        <v>1.05537477713385</v>
+        <v>1.0689026077952599</v>
       </c>
       <c r="G8">
         <v>55.5208333333333</v>
@@ -1166,29 +1204,30 @@
         <v>0.44035281996381798</v>
       </c>
       <c r="J8">
+        <v>-117.81553333050999</v>
+      </c>
+      <c r="K8">
         <v>0.34169991599597399</v>
       </c>
-      <c r="K8">
-        <v>5.3895942835032497E-2</v>
-      </c>
       <c r="L8">
+        <v>6.6632521994723901E-2</v>
+      </c>
+      <c r="M8">
         <v>-0.82017900983651904</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A9" s="1">
         <v>45684.479050925896</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C9">
         <v>351.12894</v>
@@ -1200,7 +1239,7 @@
         <v>0.274027142180158</v>
       </c>
       <c r="F9">
-        <v>79.264098932679701</v>
+        <v>80.157590032844595</v>
       </c>
       <c r="G9">
         <v>52.302624999999999</v>
@@ -1212,29 +1251,30 @@
         <v>0.51755443495451803</v>
       </c>
       <c r="J9">
+        <v>-37.944308476774602</v>
+      </c>
+      <c r="K9">
         <v>0.37772542751245602</v>
       </c>
-      <c r="K9">
-        <v>4.3727853014475704</v>
-      </c>
       <c r="L9">
+        <v>4.3839945724240899</v>
+      </c>
+      <c r="M9">
         <v>-0.65864057105660601</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O9">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A10" s="1">
         <v>45742.4440972222</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10">
         <v>395.79908</v>
@@ -1246,7 +1286,7 @@
         <v>0.20887010627168101</v>
       </c>
       <c r="F10">
-        <v>31.8524402167807</v>
+        <v>30.854267875827599</v>
       </c>
       <c r="G10">
         <v>63.575625000000002</v>
@@ -1258,40 +1298,39 @@
         <v>1.42501020490897E-2</v>
       </c>
       <c r="J10">
+        <v>-1.7222933725408101</v>
+      </c>
+      <c r="K10">
         <v>1.28246078003676E-2</v>
       </c>
-      <c r="K10">
-        <v>3.4611139949948102</v>
-      </c>
       <c r="L10">
+        <v>3.4292750835974202</v>
+      </c>
+      <c r="M10">
         <v>-4.2509912109534902</v>
       </c>
-      <c r="M10">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N10">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O10">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A11" s="1">
         <v>45763.530902777798</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>350.41699999999997</v>
       </c>
-      <c r="M11">
-        <f t="shared" si="0"/>
-        <v>0.34487962272478007</v>
-      </c>
       <c r="N11">
-        <f t="shared" si="1"/>
-        <v>0.29237660777889274</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O11">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -1302,10 +1341,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N8"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O8"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1343,18 +1382,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45231.505902777797</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2">
         <v>714.04719999999998</v>
@@ -1366,7 +1408,7 @@
         <v>0.32324005414038398</v>
       </c>
       <c r="F2">
-        <v>28.768093258691401</v>
+        <v>29.5983506265875</v>
       </c>
       <c r="G2">
         <v>67.208513227513194</v>
@@ -1378,29 +1420,30 @@
         <v>1.02097823373577E-3</v>
       </c>
       <c r="J2">
+        <v>-8.5516770594418104E-2</v>
+      </c>
+      <c r="K2">
         <v>9.7979610448898605E-4</v>
       </c>
-      <c r="K2">
-        <v>3.35926690003491</v>
-      </c>
       <c r="L2">
+        <v>3.3877186377027302</v>
+      </c>
+      <c r="M2">
         <v>-6.8869940586010197</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45279.458796296298</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>743.79520000000002</v>
@@ -1412,7 +1455,7 @@
         <v>0.87871579907905895</v>
       </c>
       <c r="F3">
-        <v>589.47237797650905</v>
+        <v>590.96639645607604</v>
       </c>
       <c r="G3">
         <v>58.628998122065703</v>
@@ -1424,29 +1467,30 @@
         <v>0.200053915250054</v>
       </c>
       <c r="J3">
+        <v>-5.2084582768903598</v>
+      </c>
+      <c r="K3">
         <v>0.16449777024491999</v>
       </c>
-      <c r="K3">
-        <v>6.3792278621815797</v>
-      </c>
       <c r="L3">
+        <v>6.38175915700121</v>
+      </c>
+      <c r="M3">
         <v>-1.6091683725129799</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M8" si="0">AVERAGE(I:I)</f>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N8" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45296.610069444403</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>456.12386666666703</v>
@@ -1458,7 +1502,7 @@
         <v>0.422753905123254</v>
       </c>
       <c r="F4">
-        <v>64.624768581672697</v>
+        <v>66.030556631691098</v>
       </c>
       <c r="G4">
         <v>54.832595600676797</v>
@@ -1470,29 +1514,30 @@
         <v>1.5919612545879001E-3</v>
       </c>
       <c r="J4">
+        <v>-7.97148872607817E-2</v>
+      </c>
+      <c r="K4">
         <v>1.2190181706383399E-3</v>
       </c>
-      <c r="K4">
-        <v>4.1685977518809496</v>
-      </c>
       <c r="L4">
+        <v>4.1901176141526397</v>
+      </c>
+      <c r="M4">
         <v>-6.4427885294265197</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45569.462962963</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5">
         <v>395.82371999999998</v>
@@ -1504,7 +1549,7 @@
         <v>0.39510332832113498</v>
       </c>
       <c r="F5">
-        <v>52.727192086974298</v>
+        <v>53.967789757068701</v>
       </c>
       <c r="G5">
         <v>75.436222222222199</v>
@@ -1516,29 +1561,30 @@
         <v>0.21503761105255101</v>
       </c>
       <c r="J5">
+        <v>-17.136375299226099</v>
+      </c>
+      <c r="K5">
         <v>0.23707665961172</v>
       </c>
-      <c r="K5">
-        <v>3.9651313013559601</v>
-      </c>
       <c r="L5">
+        <v>3.9883873826155298</v>
+      </c>
+      <c r="M5">
         <v>-1.5369423310257</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45590.473611111098</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6">
         <v>411.06707999999998</v>
@@ -1550,7 +1596,7 @@
         <v>0.363585946262801</v>
       </c>
       <c r="F6">
-        <v>41.014586930914497</v>
+        <v>42.070301544137799</v>
       </c>
       <c r="G6">
         <v>68.4775833333333</v>
@@ -1562,29 +1608,30 @@
         <v>3.1531697631642701E-2</v>
       </c>
       <c r="J6">
+        <v>-2.4052938693316901</v>
+      </c>
+      <c r="K6">
         <v>3.0937090530974799E-2</v>
       </c>
-      <c r="K6">
-        <v>3.71392778223283</v>
-      </c>
       <c r="L6">
+        <v>3.7393420652529401</v>
+      </c>
+      <c r="M6">
         <v>-3.4567619650844601</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45639.526967592603</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>365.80829999999997</v>
@@ -1596,7 +1643,7 @@
         <v>0.11668969198078299</v>
       </c>
       <c r="F7">
-        <v>1.35927936760901</v>
+        <v>1.4351821937048901</v>
       </c>
       <c r="G7">
         <v>54.87</v>
@@ -1608,29 +1655,30 @@
         <v>0.15210983764305899</v>
       </c>
       <c r="J7">
+        <v>-27.625069180142699</v>
+      </c>
+      <c r="K7">
         <v>0.11659482634669301</v>
       </c>
-      <c r="K7">
-        <v>0.30695468255557801</v>
-      </c>
       <c r="L7">
+        <v>0.36129180540658501</v>
+      </c>
+      <c r="M7">
         <v>-1.88315240302439</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>8.9110816575696306E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45684.528587963003</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C8">
         <v>329.19088799999997</v>
@@ -1642,7 +1690,7 @@
         <v>0.51440368670947101</v>
       </c>
       <c r="F8">
-        <v>117.025266996404</v>
+        <v>118.961200714924</v>
       </c>
       <c r="G8">
         <v>52.1867083333333</v>
@@ -1654,21 +1702,22 @@
         <v>2.0436212997519201E-2</v>
       </c>
       <c r="J8">
+        <v>-0.79604788901283996</v>
+      </c>
+      <c r="K8">
         <v>1.4878933413551501E-2</v>
       </c>
-      <c r="K8">
-        <v>4.7623898687165704</v>
-      </c>
       <c r="L8">
+        <v>4.77879739553509</v>
+      </c>
+      <c r="M8">
         <v>-3.8904468049059702</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>8.8826030580449938E-2</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>8.9110816575696306E-2</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -1679,10 +1728,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q16"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1720,18 +1769,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45266.452662037002</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C2">
         <v>409.7124</v>
@@ -1743,7 +1795,7 @@
         <v>0.20071662604863699</v>
       </c>
       <c r="F2">
-        <v>126.53856877099599</v>
+        <v>125.515592684373</v>
       </c>
       <c r="G2">
         <v>62.968666666666699</v>
@@ -1755,29 +1807,34 @@
         <v>3.7932408519058297E-2</v>
       </c>
       <c r="J2">
+        <v>-4.7139949011966698</v>
+      </c>
+      <c r="K2">
         <v>3.3764745220472098E-2</v>
       </c>
-      <c r="K2">
-        <v>4.8405471531679396</v>
-      </c>
       <c r="L2">
+        <v>4.8324299953511298</v>
+      </c>
+      <c r="M2">
         <v>-3.2719494262448898</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+      <c r="Q2">
+        <f>AVERAGE(K1:K16)</f>
+        <v>0.41851066083045541</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45279.417939814797</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C3">
         <v>444.28</v>
@@ -1789,7 +1846,7 @@
         <v>0.75658739105356998</v>
       </c>
       <c r="F3">
-        <v>486.50833081461201</v>
+        <v>480.18930775924503</v>
       </c>
       <c r="G3">
         <v>59.392708333333303</v>
@@ -1801,29 +1858,30 @@
         <v>6.6934508597743303E-2</v>
       </c>
       <c r="J3">
+        <v>-2.05580908822881</v>
+      </c>
+      <c r="K3">
         <v>5.58319172827028E-2</v>
       </c>
-      <c r="K3">
-        <v>6.1872540254560402</v>
-      </c>
       <c r="L3">
+        <v>6.1741804173152799</v>
+      </c>
+      <c r="M3">
         <v>-2.7040406212555999</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M16" si="0">AVERAGE(I:I)</f>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N16" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45296.400694444397</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>426.60744999999997</v>
@@ -1835,7 +1893,7 @@
         <v>0.285012367816944</v>
       </c>
       <c r="F4">
-        <v>180.62249394423401</v>
+        <v>178.927969505135</v>
       </c>
       <c r="G4">
         <v>54.871041666666699</v>
@@ -1847,29 +1905,30 @@
         <v>5.6304595414703E-2</v>
       </c>
       <c r="J4">
+        <v>-4.1865733146155897</v>
+      </c>
+      <c r="K4">
         <v>4.31584480439927E-2</v>
       </c>
-      <c r="K4">
-        <v>5.1964091844132598</v>
-      </c>
       <c r="L4">
+        <v>5.1869833198548898</v>
+      </c>
+      <c r="M4">
         <v>-2.8769791234605502</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45442.334837962997</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>892.51250000000005</v>
@@ -1881,7 +1940,7 @@
         <v>3.8657298433478003E-2</v>
       </c>
       <c r="F5">
-        <v>23.785233645707201</v>
+        <v>23.737148934319698</v>
       </c>
       <c r="G5">
         <v>72.257625000000004</v>
@@ -1893,29 +1952,30 @@
         <v>3.09288241918769E-2</v>
       </c>
       <c r="J5">
+        <v>-23.794884995299402</v>
+      </c>
+      <c r="K5">
         <v>3.23566680786452E-2</v>
       </c>
-      <c r="K5">
-        <v>3.1690649530736299</v>
-      </c>
       <c r="L5">
+        <v>3.1670412865322399</v>
+      </c>
+      <c r="M5">
         <v>-3.4760667081426702</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45484.417592592603</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C6">
         <v>2034.8627879999999</v>
@@ -1927,7 +1987,7 @@
         <v>0.31670942796431001</v>
       </c>
       <c r="F6">
-        <v>201.03278335540099</v>
+        <v>199.066611578417</v>
       </c>
       <c r="G6">
         <v>76.579041666666697</v>
@@ -1939,29 +1999,30 @@
         <v>4.9854762303598699E-2</v>
       </c>
       <c r="J6">
+        <v>-5.0588388639894299</v>
+      </c>
+      <c r="K6">
         <v>5.60087554457162E-2</v>
       </c>
-      <c r="K6">
-        <v>5.3034679960301601</v>
-      </c>
       <c r="L6">
+        <v>5.29363950026422</v>
+      </c>
+      <c r="M6">
         <v>-2.9986412544672598</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45502.410763888904</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>1722.98714</v>
@@ -1973,7 +2034,7 @@
         <v>0.47694777291652501</v>
       </c>
       <c r="F7">
-        <v>304.59536066895402</v>
+        <v>301.15616574912201</v>
       </c>
       <c r="G7">
         <v>76.361791666666704</v>
@@ -1985,29 +2046,30 @@
         <v>2.3454575425552002E-2</v>
       </c>
       <c r="J7">
+        <v>-1.5743410213597999</v>
+      </c>
+      <c r="K7">
         <v>2.6257155135099901E-2</v>
       </c>
-      <c r="K7">
-        <v>5.71898420944866</v>
-      </c>
       <c r="L7">
+        <v>5.7076289532934998</v>
+      </c>
+      <c r="M7">
         <v>-3.7526896890260999</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45569.336458333302</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>520.15418799999998</v>
@@ -2019,7 +2081,7 @@
         <v>0.13001805807807401</v>
       </c>
       <c r="F8">
-        <v>81.441506230339598</v>
+        <v>80.913576872166303</v>
       </c>
       <c r="G8">
         <v>75.600666666666697</v>
@@ -2031,29 +2093,30 @@
         <v>5.2086852237835102E-3</v>
       </c>
       <c r="J8">
+        <v>-1.2650070317995099</v>
+      </c>
+      <c r="K8">
         <v>5.7577800276754501E-3</v>
       </c>
-      <c r="K8">
-        <v>4.3998850476009697</v>
-      </c>
       <c r="L8">
+        <v>4.3933816328782704</v>
+      </c>
+      <c r="M8">
         <v>-5.2574278113436197</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A9" s="1">
         <v>45590.352199074099</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C9">
         <v>551.09719199999995</v>
@@ -2065,7 +2128,7 @@
         <v>5.6975516888096697E-2</v>
       </c>
       <c r="F9">
-        <v>35.252642693858398</v>
+        <v>35.132159403536903</v>
       </c>
       <c r="G9">
         <v>69.506833333333304</v>
@@ -2077,29 +2140,30 @@
         <v>2.05761348096275E-2</v>
       </c>
       <c r="J9">
+        <v>-10.210021026820501</v>
+      </c>
+      <c r="K9">
         <v>2.05466990492898E-2</v>
       </c>
-      <c r="K9">
-        <v>3.5625404964867</v>
-      </c>
       <c r="L9">
+        <v>3.55911693331934</v>
+      </c>
+      <c r="M9">
         <v>-3.8836233791585602</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O9">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A10" s="1">
         <v>45597.357986111099</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>628.45452</v>
@@ -2111,7 +2175,7 @@
         <v>4.2176871323439502E-2</v>
       </c>
       <c r="F10">
-        <v>25.980004093593902</v>
+        <v>25.9201818675844</v>
       </c>
       <c r="G10">
         <v>69.6570416666667</v>
@@ -2119,30 +2183,34 @@
       <c r="H10">
         <v>1.6433163391097401</v>
       </c>
+      <c r="I10">
+        <v>1.64162808869427</v>
+      </c>
       <c r="J10">
+        <v>1103.3518731004101</v>
+      </c>
+      <c r="K10">
         <v>1.6433163391097401</v>
       </c>
-      <c r="K10">
-        <v>3.25732716880957</v>
-      </c>
       <c r="L10">
+        <v>3.25502188795577</v>
+      </c>
+      <c r="M10">
         <v>0.49568848640730401</v>
       </c>
-      <c r="M10">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N10">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O10">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A11" s="1">
         <v>45618.398726851898</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>3118.5123840000001</v>
@@ -2154,7 +2222,7 @@
         <v>3.4511311120524399E-2</v>
       </c>
       <c r="F11">
-        <v>21.1939138978648</v>
+        <v>21.1611633589551</v>
       </c>
       <c r="G11">
         <v>62.832875000000001</v>
@@ -2166,29 +2234,30 @@
         <v>0.63468059732398197</v>
       </c>
       <c r="J11">
+        <v>457.595214036014</v>
+      </c>
+      <c r="K11">
         <v>0.56366732080101301</v>
       </c>
-      <c r="K11">
-        <v>3.0537140601731299</v>
-      </c>
       <c r="L11">
+        <v>3.0521675846354701</v>
+      </c>
+      <c r="M11">
         <v>-0.45463340297472599</v>
       </c>
-      <c r="M11">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N11">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O11">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A12" s="1">
         <v>45635.392824074101</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C12">
         <v>2329.1665200000002</v>
@@ -2200,7 +2269,7 @@
         <v>3.9109156854677397E-2</v>
       </c>
       <c r="F12">
-        <v>24.062123859764501</v>
+        <v>24.0137761154011</v>
       </c>
       <c r="G12">
         <v>56.872333333333302</v>
@@ -2208,30 +2277,34 @@
       <c r="H12">
         <v>2.152726136449</v>
       </c>
+      <c r="I12">
+        <v>2.70467538288039</v>
+      </c>
       <c r="J12">
+        <v>1526.9804203271599</v>
+      </c>
+      <c r="K12">
         <v>2.152726136449</v>
       </c>
-      <c r="K12">
-        <v>3.1806389801238302</v>
-      </c>
       <c r="L12">
+        <v>3.1786276704785799</v>
+      </c>
+      <c r="M12">
         <v>0.99498189876823395</v>
       </c>
-      <c r="M12">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N12">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O12">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A13" s="1">
         <v>45660.411574074104</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C13">
         <v>552.81111999999996</v>
@@ -2243,7 +2316,7 @@
         <v>5.9249035421147699E-2</v>
       </c>
       <c r="F13">
-        <v>36.681435442351599</v>
+        <v>36.550549878520599</v>
       </c>
       <c r="G13">
         <v>58.6762916666667</v>
@@ -2255,29 +2328,30 @@
         <v>0.84133921279000901</v>
       </c>
       <c r="J13">
+        <v>-325.21801263957502</v>
+      </c>
+      <c r="K13">
         <v>0.69249876487298101</v>
       </c>
-      <c r="K13">
-        <v>3.6022707808196901</v>
-      </c>
       <c r="L13">
+        <v>3.5986962306385899</v>
+      </c>
+      <c r="M13">
         <v>-0.17276035575285201</v>
       </c>
-      <c r="M13">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N13">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O13">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A14" s="1">
         <v>45684.409837963001</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14">
         <v>560.08052399999997</v>
@@ -2289,7 +2363,7 @@
         <v>0.216853459021603</v>
       </c>
       <c r="F14">
-        <v>136.86948922984999</v>
+        <v>135.72378343994899</v>
       </c>
       <c r="G14">
         <v>53.521625</v>
@@ -2301,29 +2375,30 @@
         <v>0.17242135645319001</v>
       </c>
       <c r="J14">
+        <v>-16.385838425175901</v>
+      </c>
+      <c r="K14">
         <v>0.12881644181349999</v>
       </c>
-      <c r="K14">
-        <v>4.9190278384258299</v>
-      </c>
       <c r="L14">
+        <v>4.9106218163322897</v>
+      </c>
+      <c r="M14">
         <v>-1.7578140510860201</v>
       </c>
-      <c r="M14">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N14">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O14">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A15" s="1">
         <v>45742.371412036999</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C15">
         <v>335.30592000000001</v>
@@ -2335,7 +2410,7 @@
         <v>0.106979611271476</v>
       </c>
       <c r="F15">
-        <v>66.816132668238495</v>
+        <v>66.431348555876397</v>
       </c>
       <c r="G15">
         <v>63.225333333333303</v>
@@ -2347,29 +2422,30 @@
         <v>0.59835790323903604</v>
       </c>
       <c r="J15">
+        <v>-140.25575841804701</v>
+      </c>
+      <c r="K15">
         <v>0.53520797229477701</v>
       </c>
-      <c r="K15">
-        <v>4.2019445583940396</v>
-      </c>
       <c r="L15">
+        <v>4.19616906187568</v>
+      </c>
+      <c r="M15">
         <v>-0.51356620366171402</v>
       </c>
-      <c r="M15">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N15">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O15">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.75">
       <c r="A16" s="1">
         <v>45763.334143518499</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C16">
         <v>354.50755500000002</v>
@@ -2380,6 +2456,9 @@
       <c r="E16">
         <v>6.0014183168862097E-2</v>
       </c>
+      <c r="F16">
+        <v>37.027075296500897</v>
+      </c>
       <c r="G16">
         <v>65.204999999999998</v>
       </c>
@@ -2390,18 +2469,22 @@
         <v>0.310539122154604</v>
       </c>
       <c r="J16">
+        <v>-134.84409761732499</v>
+      </c>
+      <c r="K16">
         <v>0.28774476883222599</v>
       </c>
       <c r="L16">
+        <v>3.6116494098052199</v>
+      </c>
+      <c r="M16">
         <v>-1.16944538826829</v>
       </c>
-      <c r="M16">
-        <f t="shared" si="0"/>
-        <v>0.21911789895744341</v>
-      </c>
       <c r="N16">
-        <f t="shared" si="1"/>
-        <v>0.27515513148828169</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O16">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -2412,10 +2495,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2453,18 +2536,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45231.413888888899</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>434.69794999999999</v>
@@ -2476,7 +2562,7 @@
         <v>0.45326953896332001</v>
       </c>
       <c r="F2">
-        <v>14.1949526530613</v>
+        <v>14.1100368821192</v>
       </c>
       <c r="G2">
         <v>67.299833333333297</v>
@@ -2488,29 +2574,30 @@
         <v>1.27094099773852E-2</v>
       </c>
       <c r="J2">
+        <v>-0.76044828481318405</v>
+      </c>
+      <c r="K2">
         <v>1.2215882003802799E-2</v>
       </c>
-      <c r="K2">
-        <v>2.6528864544534501</v>
-      </c>
       <c r="L2">
+        <v>2.6468863797606099</v>
+      </c>
+      <c r="M2">
         <v>-4.3654126167792198</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>0.10592607582249888</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>0.10053694390274144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45296.434953703698</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C3">
         <v>618.29094999999995</v>
@@ -2522,7 +2609,7 @@
         <v>0.52599051773861105</v>
       </c>
       <c r="F3">
-        <v>23.486515987919301</v>
+        <v>23.639121954740101</v>
       </c>
       <c r="G3">
         <v>55.262291666666698</v>
@@ -2534,29 +2621,30 @@
         <v>2.95461493180833E-2</v>
       </c>
       <c r="J3">
+        <v>-1.19973709296109</v>
+      </c>
+      <c r="K3">
         <v>2.2810224388765399E-2</v>
       </c>
-      <c r="K3">
-        <v>3.1564264687228101</v>
-      </c>
       <c r="L3">
+        <v>3.1629030494936199</v>
+      </c>
+      <c r="M3">
         <v>-3.5218018543459699</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M6" si="0">AVERAGE(I:I)</f>
-        <v>0.10592607582249888</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N6" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>0.10053694390274144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45569.400115740696</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C4">
         <v>555.11051999999995</v>
@@ -2568,7 +2656,7 @@
         <v>0.48690939353906698</v>
       </c>
       <c r="F4">
-        <v>18.0792633709287</v>
+        <v>18.078880049837199</v>
       </c>
       <c r="G4">
         <v>75.319166666666703</v>
@@ -2580,29 +2668,30 @@
         <v>0.114810057389193</v>
       </c>
       <c r="J4">
+        <v>-7.4098749215135902</v>
+      </c>
+      <c r="K4">
         <v>0.126352936677328</v>
       </c>
-      <c r="K4">
-        <v>2.8947656113756599</v>
-      </c>
       <c r="L4">
+        <v>2.89474440889924</v>
+      </c>
+      <c r="M4">
         <v>-2.1644761910142201</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>0.10592607582249888</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>0.10053694390274144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45590.382638888899</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C5">
         <v>921.71709999999996</v>
@@ -2614,7 +2703,7 @@
         <v>0.45046535211951499</v>
       </c>
       <c r="F5">
-        <v>13.881694135153399</v>
+        <v>13.7903622475802</v>
       </c>
       <c r="G5">
         <v>68.263083333333299</v>
@@ -2622,30 +2711,34 @@
       <c r="H5">
         <v>-0.62628271367326904</v>
       </c>
+      <c r="I5">
+        <v>0.64070198635915099</v>
+      </c>
       <c r="J5">
+        <v>-39.2881153687024</v>
+      </c>
+      <c r="K5">
         <v>0.62628271367326904</v>
       </c>
-      <c r="K5">
-        <v>2.63057100347724</v>
-      </c>
       <c r="L5">
+        <v>2.6239699603202502</v>
+      </c>
+      <c r="M5">
         <v>-0.44519085004674103</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>0.10592607582249888</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>0.10053694390274144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45684.449305555601</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>438.31808999999998</v>
@@ -2657,7 +2750,7 @@
         <v>0.51969792065458198</v>
       </c>
       <c r="F6">
-        <v>22.550048418024101</v>
+        <v>22.6737312584969</v>
       </c>
       <c r="G6">
         <v>53.172249999999998</v>
@@ -2669,21 +2762,22 @@
         <v>0.26663868660533402</v>
       </c>
       <c r="J6">
+        <v>-10.4946666210505</v>
+      </c>
+      <c r="K6">
         <v>0.197842978098901</v>
       </c>
-      <c r="K6">
-        <v>3.1157372130871401</v>
-      </c>
       <c r="L6">
+        <v>3.1212070411169899</v>
+      </c>
+      <c r="M6">
         <v>-1.32186077071735</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.10592607582249888</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>0.10053694390274144</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -2694,10 +2788,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2735,18 +2829,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45266.611111111102</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>615.23294999999996</v>
@@ -2758,7 +2855,7 @@
         <v>0.234268725880109</v>
       </c>
       <c r="F2">
-        <v>28.539624448278001</v>
+        <v>28.445732115260999</v>
       </c>
       <c r="G2">
         <v>63.182749999999999</v>
@@ -2770,29 +2867,30 @@
         <v>1.0333831699921499E-2</v>
       </c>
       <c r="J2">
+        <v>-1.10496470250395</v>
+      </c>
+      <c r="K2">
         <v>9.2342488193686706E-3</v>
       </c>
-      <c r="K2">
-        <v>3.3512934531771799</v>
-      </c>
       <c r="L2">
+        <v>3.3479981357958501</v>
+      </c>
+      <c r="M2">
         <v>-4.5723321353034301</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45296.650231481501</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <v>612.31027500000005</v>
@@ -2804,7 +2902,7 @@
         <v>0.44772677954446899</v>
       </c>
       <c r="F3">
-        <v>187.93417675073701</v>
+        <v>187.33984571034901</v>
       </c>
       <c r="G3">
         <v>57.347416666666703</v>
@@ -2816,29 +2914,30 @@
         <v>3.4306204774390801E-2</v>
       </c>
       <c r="J3">
+        <v>-1.7080599446193601</v>
+      </c>
+      <c r="K3">
         <v>2.7545495641895699E-2</v>
       </c>
-      <c r="K3">
-        <v>5.2360917778560596</v>
-      </c>
       <c r="L3">
+        <v>5.2329243241997201</v>
+      </c>
+      <c r="M3">
         <v>-3.3724290439576099</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M16" si="0">AVERAGE(I:I)</f>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N15" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45331.457060185203</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>504.21780863999999</v>
@@ -2850,7 +2949,7 @@
         <v>0.34695286733230901</v>
       </c>
       <c r="F4">
-        <v>89.654753749752999</v>
+        <v>89.366755994949202</v>
       </c>
       <c r="G4">
         <v>56.771625</v>
@@ -2862,29 +2961,30 @@
         <v>9.9277292154952998E-2</v>
       </c>
       <c r="J4">
+        <v>-6.3040225822830003</v>
+      </c>
+      <c r="K4">
         <v>7.8857717580850806E-2</v>
       </c>
-      <c r="K4">
-        <v>4.4959662242979004</v>
-      </c>
       <c r="L4">
+        <v>4.49274875614379</v>
+      </c>
+      <c r="M4">
         <v>-2.30983841328699</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45442.515972222202</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>664.44209999999998</v>
@@ -2896,7 +2996,7 @@
         <v>5.9138536458891298E-2</v>
       </c>
       <c r="F5">
-        <v>0.53953030067585805</v>
+        <v>0.53761255781817996</v>
       </c>
       <c r="G5">
         <v>69.956999999999994</v>
@@ -2908,29 +3008,30 @@
         <v>1.19519645480923E-2</v>
       </c>
       <c r="J5">
+        <v>-5.7616663344601502</v>
+      </c>
+      <c r="K5">
         <v>1.2026837343753901E-2</v>
       </c>
-      <c r="K5">
-        <v>-0.61705633149436401</v>
-      </c>
       <c r="L5">
+        <v>-0.620617131009223</v>
+      </c>
+      <c r="M5">
         <v>-4.42685961678648</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45484.550925925898</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>20118.913499999999</v>
@@ -2942,7 +3043,7 @@
         <v>0.146682711547242</v>
       </c>
       <c r="F6">
-        <v>7.4821242321530796</v>
+        <v>7.4568488376066497</v>
       </c>
       <c r="G6">
         <v>73.537000000000006</v>
@@ -2950,30 +3051,34 @@
       <c r="H6">
         <v>1.8467246153386201</v>
       </c>
+      <c r="I6">
+        <v>1.7280533772406299</v>
+      </c>
       <c r="J6">
+        <v>358.57736745069201</v>
+      </c>
+      <c r="K6">
         <v>1.8467246153386201</v>
       </c>
-      <c r="K6">
-        <v>2.0125167399251098</v>
-      </c>
       <c r="L6">
+        <v>2.0091329171488201</v>
+      </c>
+      <c r="M6">
         <v>0.54699555951163803</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45502.5288194444</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7">
         <v>2747.5827119999999</v>
@@ -2985,7 +3090,7 @@
         <v>0.30285820571641198</v>
       </c>
       <c r="F7">
-        <v>60.429220662836499</v>
+        <v>60.233498000718598</v>
       </c>
       <c r="G7">
         <v>74.329666666666697</v>
@@ -2997,29 +3102,30 @@
         <v>0.215449086397794</v>
       </c>
       <c r="J7">
+        <v>-21.963193939423501</v>
+      </c>
+      <c r="K7">
         <v>0.23328053058185999</v>
       </c>
-      <c r="K7">
-        <v>4.1014727737627004</v>
-      </c>
       <c r="L7">
+        <v>4.09822864275122</v>
+      </c>
+      <c r="M7">
         <v>-1.5350306553665301</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45569.486458333296</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C8">
         <v>1103.890144</v>
@@ -3031,7 +3137,7 @@
         <v>0.42756115791951899</v>
       </c>
       <c r="F8">
-        <v>165.10934080357401</v>
+        <v>164.58582373578801</v>
       </c>
       <c r="G8">
         <v>75.326458333333306</v>
@@ -3043,29 +3149,30 @@
         <v>3.20015690036934E-2</v>
       </c>
       <c r="J8">
+        <v>-2.35208018663586</v>
+      </c>
+      <c r="K8">
         <v>3.5218972221151799E-2</v>
       </c>
-      <c r="K8">
-        <v>5.1066079259675599</v>
-      </c>
       <c r="L8">
+        <v>5.1034321589919598</v>
+      </c>
+      <c r="M8">
         <v>-3.4419703460189899</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A9" s="1">
         <v>45590.509490740696</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C9">
         <v>509.79309000000001</v>
@@ -3077,7 +3184,7 @@
         <v>0.37002135752523302</v>
       </c>
       <c r="F9">
-        <v>108.04415257551901</v>
+        <v>107.698437411738</v>
       </c>
       <c r="G9">
         <v>68.863500000000002</v>
@@ -3089,29 +3196,30 @@
         <v>0.19759869761570001</v>
       </c>
       <c r="J9">
+        <v>-14.9162584675987</v>
+      </c>
+      <c r="K9">
         <v>0.195137400329535</v>
       </c>
-      <c r="K9">
-        <v>4.6825399637237304</v>
-      </c>
       <c r="L9">
+        <v>4.6793350753452803</v>
+      </c>
+      <c r="M9">
         <v>-1.6215170847037499</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O9">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A10" s="1">
         <v>45597.442013888904</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C10">
         <v>709.25940000000003</v>
@@ -3123,7 +3231,7 @@
         <v>0.30001852958251402</v>
       </c>
       <c r="F10">
-        <v>58.692552936783898</v>
+        <v>58.502329278323103</v>
       </c>
       <c r="G10">
         <v>69.199291666666696</v>
@@ -3131,30 +3239,34 @@
       <c r="H10">
         <v>-2.4587062321850501</v>
       </c>
+      <c r="I10">
+        <v>2.4751540809886499</v>
+      </c>
       <c r="J10">
+        <v>-231.91580033051</v>
+      </c>
+      <c r="K10">
         <v>2.4587062321850501</v>
       </c>
-      <c r="K10">
-        <v>4.0723128522914998</v>
-      </c>
       <c r="L10">
+        <v>4.0690665701686202</v>
+      </c>
+      <c r="M10">
         <v>0.906302649027806</v>
       </c>
-      <c r="M10">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N10">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O10">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A11" s="1">
         <v>45618.515393518501</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C11">
         <v>2030.428296</v>
@@ -3166,7 +3278,7 @@
         <v>0.18724196474367</v>
       </c>
       <c r="F11">
-        <v>15.2013972009324</v>
+        <v>15.150771774911</v>
       </c>
       <c r="G11">
         <v>65.922749999999994</v>
@@ -3174,30 +3286,34 @@
       <c r="H11">
         <v>-2.6054422986912802</v>
       </c>
+      <c r="I11">
+        <v>2.7763528639902799</v>
+      </c>
       <c r="J11">
+        <v>-391.788019986856</v>
+      </c>
+      <c r="K11">
         <v>2.6054422986912802</v>
       </c>
-      <c r="K11">
-        <v>2.7213873447417201</v>
-      </c>
       <c r="L11">
+        <v>2.7180514728962102</v>
+      </c>
+      <c r="M11">
         <v>1.0211381469548899</v>
       </c>
-      <c r="M11">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N11">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O11">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A12" s="1">
         <v>45639.551041666702</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <v>526.36743999999999</v>
@@ -3209,7 +3325,7 @@
         <v>0.14840614156752799</v>
       </c>
       <c r="F12">
-        <v>7.5786622463844298</v>
+        <v>7.55305171349909</v>
       </c>
       <c r="G12">
         <v>61.354750000000003</v>
@@ -3221,29 +3337,30 @@
         <v>0.58086027463756795</v>
       </c>
       <c r="J12">
+        <v>94.590389908381596</v>
+      </c>
+      <c r="K12">
         <v>0.50225871766377705</v>
       </c>
-      <c r="K12">
-        <v>2.0253366994331801</v>
-      </c>
       <c r="L12">
+        <v>2.0219516820573902</v>
+      </c>
+      <c r="M12">
         <v>-0.54324504221023096</v>
       </c>
-      <c r="M12">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N12">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O12">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A13" s="1">
         <v>45660.526851851901</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C13">
         <v>350.63274000000001</v>
@@ -3255,7 +3372,7 @@
         <v>0.12874386448073599</v>
       </c>
       <c r="F13">
-        <v>5.0141113348335997</v>
+        <v>4.9970274005783599</v>
       </c>
       <c r="G13">
         <v>60.610833333333296</v>
@@ -3267,29 +3384,30 @@
         <v>2.90951118423101E-2</v>
       </c>
       <c r="J13">
+        <v>-5.3800167652109696</v>
+      </c>
+      <c r="K13">
         <v>2.48130778879441E-2</v>
       </c>
-      <c r="K13">
-        <v>1.6122562042828801</v>
-      </c>
       <c r="L13">
+        <v>1.6088432157527499</v>
+      </c>
+      <c r="M13">
         <v>-3.53718509684205</v>
       </c>
-      <c r="M13">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N13">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O13">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A14" s="1">
         <v>45684.584027777797</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C14">
         <v>345.56297999999998</v>
@@ -3301,7 +3419,7 @@
         <v>0.39129596301150699</v>
       </c>
       <c r="F14">
-        <v>127.14743063651601</v>
+        <v>126.741991039374</v>
       </c>
       <c r="G14">
         <v>53.251916666666702</v>
@@ -3313,29 +3431,30 @@
         <v>1.9326891841915099E-2</v>
       </c>
       <c r="J14">
+        <v>-1.01219787892574</v>
+      </c>
+      <c r="K14">
         <v>1.4364999865905699E-2</v>
       </c>
-      <c r="K14">
-        <v>4.8453472843223597</v>
-      </c>
       <c r="L14">
+        <v>4.8421534534088204</v>
+      </c>
+      <c r="M14">
         <v>-3.94625779321141</v>
       </c>
-      <c r="M14">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N14">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O14">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A15" s="1">
         <v>45742.522453703699</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C15">
         <v>342.608475</v>
@@ -3346,6 +3465,9 @@
       <c r="E15">
         <v>0.26084640141308302</v>
       </c>
+      <c r="F15">
+        <v>38.931853753656902</v>
+      </c>
       <c r="G15">
         <v>61.619416666666702</v>
       </c>
@@ -3356,33 +3478,39 @@
         <v>1.6426728788685299E-2</v>
       </c>
       <c r="J15">
+        <v>-1.53009939100035</v>
+      </c>
+      <c r="K15">
         <v>1.42738229065186E-2</v>
       </c>
       <c r="L15">
+        <v>3.6618127781012402</v>
+      </c>
+      <c r="M15">
         <v>-4.1088454666534</v>
       </c>
-      <c r="M15">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
-      </c>
       <c r="N15">
-        <f t="shared" si="1"/>
-        <v>0.16386765526403613</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O15">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A16" s="1">
         <v>45763.568518518499</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C16">
         <v>380.63817</v>
       </c>
-      <c r="M16">
-        <f t="shared" si="0"/>
-        <v>0.11332978666409303</v>
+      <c r="N16">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O16">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -3393,10 +3521,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3434,18 +3562,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45279.534722222197</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2">
         <v>811.21124999999995</v>
@@ -3456,6 +3587,9 @@
       <c r="E2">
         <v>0.58613206590049605</v>
       </c>
+      <c r="F2">
+        <v>381.085669931447</v>
+      </c>
       <c r="G2">
         <v>57.410541666666703</v>
       </c>
@@ -3466,26 +3600,30 @@
         <v>1.87415413273145E-3</v>
       </c>
       <c r="J2">
+        <v>-7.1382264927651498E-2</v>
+      </c>
+      <c r="K2">
         <v>1.5068415282105199E-3</v>
       </c>
       <c r="L2">
+        <v>5.9430242053136197</v>
+      </c>
+      <c r="M2">
         <v>-6.2795978505590497</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>0.28980508581652814</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>0.18228919660150089</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45296.649884259299</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3">
         <v>637.03409999999997</v>
@@ -3496,6 +3634,9 @@
       <c r="E3">
         <v>0.23937442308451001</v>
       </c>
+      <c r="F3">
+        <v>14.115024666976799</v>
+      </c>
       <c r="G3">
         <v>52.158749999999998</v>
       </c>
@@ -3506,26 +3647,30 @@
         <v>0.45342657131430503</v>
       </c>
       <c r="J3">
+        <v>-37.941017984035199</v>
+      </c>
+      <c r="K3">
         <v>0.33001104403172099</v>
       </c>
       <c r="L3">
+        <v>2.6472398092757898</v>
+      </c>
+      <c r="M3">
         <v>-0.79092193805088995</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M6" si="0">AVERAGE(I:I)</f>
-        <v>0.28980508581652814</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N6" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>0.18228919660150089</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45502.510416666701</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>718.57919000000004</v>
@@ -3536,6 +3681,9 @@
       <c r="E4">
         <v>0.29234008845640103</v>
       </c>
+      <c r="F4">
+        <v>29.540841265125199</v>
+      </c>
       <c r="G4">
         <v>76.433750000000003</v>
       </c>
@@ -3546,26 +3694,30 @@
         <v>0.44003583756701897</v>
       </c>
       <c r="J4">
+        <v>-48.2498856951741</v>
+      </c>
+      <c r="K4">
         <v>0.49319429387923502</v>
       </c>
       <c r="L4">
+        <v>3.3857737555442098</v>
+      </c>
+      <c r="M4">
         <v>-0.82089910637066998</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>0.28980508581652814</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>0.18228919660150089</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45590.492476851898</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C5">
         <v>505.04641199999998</v>
@@ -3576,6 +3728,9 @@
       <c r="E5">
         <v>0.23014485917083699</v>
       </c>
+      <c r="F5">
+        <v>12.2253507682329</v>
+      </c>
       <c r="G5">
         <v>67.998583333333301</v>
       </c>
@@ -3586,26 +3741,30 @@
         <v>0.263883780252057</v>
       </c>
       <c r="J5">
+        <v>-31.5116940071653</v>
+      </c>
+      <c r="K5">
         <v>0.256744343569899</v>
       </c>
       <c r="L5">
+        <v>2.50351172764729</v>
+      </c>
+      <c r="M5">
         <v>-1.3322464990818399</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>0.28980508581652814</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>0.18228919660150089</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45684.6167824074</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>450.50428799999997</v>
@@ -3616,25 +3775,35 @@
       <c r="E6">
         <v>0.30386676206507501</v>
       </c>
+      <c r="F6">
+        <v>33.974307377583699</v>
+      </c>
       <c r="G6">
         <v>49.510666666666701</v>
       </c>
       <c r="H6">
         <v>-1.09548953548564</v>
       </c>
+      <c r="I6">
+        <v>1.58388781907339</v>
+      </c>
       <c r="J6">
+        <v>-98.775054541475498</v>
+      </c>
+      <c r="K6">
         <v>1.09548953548564</v>
       </c>
       <c r="L6">
+        <v>3.5256045735919899</v>
+      </c>
+      <c r="M6">
         <v>0.459882469592234</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.28980508581652814</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>0.18228919660150089</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -3645,10 +3814,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O9"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3686,18 +3855,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45231.5222222222</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C2">
         <v>744.31614999999999</v>
@@ -3709,7 +3881,7 @@
         <v>0.13055244711888001</v>
       </c>
       <c r="F2">
-        <v>1.9348746162310799</v>
+        <v>5.0350457016229999</v>
       </c>
       <c r="G2">
         <v>68.842375000000004</v>
@@ -3721,29 +3893,30 @@
         <v>2.02631658657456E-2</v>
       </c>
       <c r="J2">
+        <v>-4.3338981527661797</v>
+      </c>
+      <c r="K2">
         <v>2.00045800791511E-2</v>
       </c>
-      <c r="K2">
-        <v>0.66004252656888096</v>
-      </c>
       <c r="L2">
+        <v>1.6164226029164199</v>
+      </c>
+      <c r="M2">
         <v>-3.89895053048641</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45279.418749999997</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>452.6567</v>
@@ -3755,7 +3928,7 @@
         <v>0.72138680186451298</v>
       </c>
       <c r="F3">
-        <v>743.27851864173499</v>
+        <v>848.07575662464205</v>
       </c>
       <c r="G3">
         <v>60.173708333333302</v>
@@ -3767,29 +3940,30 @@
         <v>2.11178428187733E-2</v>
       </c>
       <c r="J3">
+        <v>-0.69090866053144095</v>
+      </c>
+      <c r="K3">
         <v>1.7867765253196301E-2</v>
       </c>
-      <c r="K3">
-        <v>6.6110708313294202</v>
-      </c>
       <c r="L3">
+        <v>6.7429699674439796</v>
+      </c>
+      <c r="M3">
         <v>-3.85763696462327</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M9" si="0">AVERAGE(I:I)</f>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N9" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45296.551157407397</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>669.22050000000002</v>
@@ -3801,7 +3975,7 @@
         <v>0.23229443381963699</v>
       </c>
       <c r="F4">
-        <v>14.448294498683101</v>
+        <v>28.4358935594237</v>
       </c>
       <c r="G4">
         <v>57.088374999999999</v>
@@ -3813,29 +3987,30 @@
         <v>2.2110586942343101E-2</v>
       </c>
       <c r="J4">
+        <v>-2.1109281647562002</v>
+      </c>
+      <c r="K4">
         <v>1.7669774219275299E-2</v>
       </c>
-      <c r="K4">
-        <v>2.6705763798198201</v>
-      </c>
       <c r="L4">
+        <v>3.3476522048974702</v>
+      </c>
+      <c r="M4">
         <v>-3.81169873800004</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45569.448379629597</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C5">
         <v>373.09719000000001</v>
@@ -3847,7 +4022,7 @@
         <v>0.253452518093848</v>
       </c>
       <c r="F5">
-        <v>19.4830675459072</v>
+        <v>36.817077025390901</v>
       </c>
       <c r="G5">
         <v>76.006291666666698</v>
@@ -3859,29 +4034,30 @@
         <v>0.22266258013392901</v>
       </c>
       <c r="J5">
+        <v>-27.9458373309221</v>
+      </c>
+      <c r="K5">
         <v>0.247807878923372</v>
       </c>
-      <c r="K5">
-        <v>2.9695457573728601</v>
-      </c>
       <c r="L5">
+        <v>3.6059617871401799</v>
+      </c>
+      <c r="M5">
         <v>-1.50209774697395</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45590.450462963003</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6">
         <v>441.72498000000002</v>
@@ -3893,7 +4069,7 @@
         <v>0.20831663046725299</v>
       </c>
       <c r="F6">
-        <v>9.8345107413557908</v>
+        <v>20.4335550955565</v>
       </c>
       <c r="G6">
         <v>69.406999999999996</v>
@@ -3905,29 +4081,30 @@
         <v>5.1376184809108202E-2</v>
       </c>
       <c r="J6">
+        <v>-6.9585096100707302</v>
+      </c>
+      <c r="K6">
         <v>5.1208046458898503E-2</v>
       </c>
-      <c r="K6">
-        <v>2.2858977039188999</v>
-      </c>
       <c r="L6">
+        <v>3.0171784071787799</v>
+      </c>
+      <c r="M6">
         <v>-2.9685805444538902</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45684.551504629599</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C7">
         <v>395.99175600000001</v>
@@ -3939,7 +4116,7 @@
         <v>0.32786079628103298</v>
       </c>
       <c r="F7">
-        <v>47.780668829864602</v>
+        <v>79.726341875144499</v>
       </c>
       <c r="G7">
         <v>52.709458333333302</v>
@@ -3947,30 +4124,34 @@
       <c r="H7">
         <v>-0.55263832284044401</v>
       </c>
+      <c r="I7">
+        <v>0.75123960858564598</v>
+      </c>
       <c r="J7">
+        <v>-46.432245470366297</v>
+      </c>
+      <c r="K7">
         <v>0.55263832284044401</v>
       </c>
-      <c r="K7">
-        <v>3.86662113991322</v>
-      </c>
       <c r="L7">
+        <v>4.3786000440513702</v>
+      </c>
+      <c r="M7">
         <v>-0.286030625393914</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45742.479282407403</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8">
         <v>362.407284</v>
@@ -3982,7 +4163,7 @@
         <v>0.199539004922166</v>
       </c>
       <c r="F8">
-        <v>8.4491882225159092</v>
+        <v>17.958644231798001</v>
       </c>
       <c r="G8">
         <v>63.168416666666701</v>
@@ -3994,40 +4175,39 @@
         <v>7.0213185906546002E-2</v>
       </c>
       <c r="J8">
+        <v>-8.8143890125182107</v>
+      </c>
+      <c r="K8">
         <v>6.2742073597595302E-2</v>
       </c>
-      <c r="K8">
-        <v>2.1340703684129099</v>
-      </c>
       <c r="L8">
+        <v>2.8880715718174401</v>
+      </c>
+      <c r="M8">
         <v>-2.6562191521622802</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A9" s="1">
         <v>45763.530902777798</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C9">
         <v>350.41699999999997</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="0"/>
-        <v>6.7957257746074209E-2</v>
-      </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>7.162905879313583E-2</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O9">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>
@@ -4038,10 +4218,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:N13"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O13"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4079,18 +4259,21 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>45266.638425925899</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2">
         <v>711.255675</v>
@@ -4102,7 +4285,7 @@
         <v>9.2948582820242806E-2</v>
       </c>
       <c r="F2">
-        <v>1.8507918811930499</v>
+        <v>22.1394967157139</v>
       </c>
       <c r="G2">
         <v>57.605125000000001</v>
@@ -4114,29 +4297,30 @@
         <v>8.3953767192955202E-3</v>
       </c>
       <c r="J2">
+        <v>-2.0245490857211998</v>
+      </c>
+      <c r="K2">
         <v>6.7749825617792999E-3</v>
       </c>
-      <c r="K2">
-        <v>0.61561359139371596</v>
-      </c>
       <c r="L2">
+        <v>3.0973631951212099</v>
+      </c>
+      <c r="M2">
         <v>-4.7800741152134103</v>
       </c>
-      <c r="M2">
-        <f>AVERAGE(I:I)</f>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N2">
-        <f>_xlfn.STDEV.P(I:I)</f>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O2">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
         <v>45296.691319444399</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>680.57703333333302</v>
@@ -4148,7 +4332,7 @@
         <v>0.304619300450722</v>
       </c>
       <c r="F3">
-        <v>64.160963220889599</v>
+        <v>194.27305049863901</v>
       </c>
       <c r="G3">
         <v>52.267458333333302</v>
@@ -4160,29 +4344,30 @@
         <v>5.6427577340035402E-2</v>
       </c>
       <c r="J3">
+        <v>-3.7187084560364001</v>
+      </c>
+      <c r="K3">
         <v>4.1153993632000299E-2</v>
       </c>
-      <c r="K3">
-        <v>4.16139497623998</v>
-      </c>
       <c r="L3">
+        <v>5.2692646462933901</v>
+      </c>
+      <c r="M3">
         <v>-2.8747972800503701</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M13" si="0">AVERAGE(I:I)</f>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N3">
-        <f t="shared" ref="N3:N13" si="1">_xlfn.STDEV.P(I:I)</f>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O3">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A4" s="1">
         <v>45331.513657407399</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4">
         <v>464.2354962</v>
@@ -4194,7 +4379,7 @@
         <v>0.26214009253193299</v>
       </c>
       <c r="F4">
-        <v>41.006683216447897</v>
+        <v>147.63081525566301</v>
       </c>
       <c r="G4">
         <v>55.680374999999998</v>
@@ -4202,30 +4387,34 @@
       <c r="H4">
         <v>-1.4668428620366101</v>
       </c>
+      <c r="I4">
+        <v>1.88456765595585</v>
+      </c>
       <c r="J4">
+        <v>-154.91802860734899</v>
+      </c>
+      <c r="K4">
         <v>1.4668428620366101</v>
       </c>
-      <c r="K4">
-        <v>3.7137350586996098</v>
-      </c>
       <c r="L4">
+        <v>4.9947146658206902</v>
+      </c>
+      <c r="M4">
         <v>0.63369843435726703</v>
       </c>
-      <c r="M4">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O4">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A5" s="1">
         <v>45502.6175925926</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>703.29944999999998</v>
@@ -4237,7 +4426,7 @@
         <v>0.14969712289074899</v>
       </c>
       <c r="F5">
-        <v>7.7407951713826604</v>
+        <v>53.049521358984101</v>
       </c>
       <c r="G5">
         <v>77.678708333333304</v>
@@ -4249,29 +4438,30 @@
         <v>0.100544975455905</v>
       </c>
       <c r="J5">
+        <v>-22.0081778872851</v>
+      </c>
+      <c r="K5">
         <v>0.11499012465521399</v>
       </c>
-      <c r="K5">
-        <v>2.0465044176454801</v>
-      </c>
       <c r="L5">
+        <v>3.9712258425684701</v>
+      </c>
+      <c r="M5">
         <v>-2.2971501346146801</v>
       </c>
-      <c r="M5">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O5">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A6" s="1">
         <v>45569.557407407403</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>403.84739999999999</v>
@@ -4283,7 +4473,7 @@
         <v>0.19368252554686899</v>
       </c>
       <c r="F6">
-        <v>16.600096724586301</v>
+        <v>84.849376312328204</v>
       </c>
       <c r="G6">
         <v>76.782666666666699</v>
@@ -4295,29 +4485,30 @@
         <v>2.5267627188960799E-2</v>
       </c>
       <c r="J6">
+        <v>-4.2072892663145502</v>
+      </c>
+      <c r="K6">
         <v>2.8478304234839501E-2</v>
       </c>
-      <c r="K6">
-        <v>2.8094085221278302</v>
-      </c>
       <c r="L6">
+        <v>4.4408776411797799</v>
+      </c>
+      <c r="M6">
         <v>-3.6782312603302598</v>
       </c>
-      <c r="M6">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O6">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A7" s="1">
         <v>45590.536805555603</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C7">
         <v>385.73862000000003</v>
@@ -4329,7 +4520,7 @@
         <v>0.189070453385662</v>
       </c>
       <c r="F7">
-        <v>15.4378007004605</v>
+        <v>81.176183245272497</v>
       </c>
       <c r="G7">
         <v>67.770875000000004</v>
@@ -4341,29 +4532,30 @@
         <v>1.8288066770139E-2</v>
       </c>
       <c r="J7">
+        <v>-2.6466005264160199</v>
+      </c>
+      <c r="K7">
         <v>1.7721333548753701E-2</v>
       </c>
-      <c r="K7">
-        <v>2.7368190927708298</v>
-      </c>
       <c r="L7">
+        <v>4.3966218943566204</v>
+      </c>
+      <c r="M7">
         <v>-4.0015065209007501</v>
       </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N7">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O7">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A8" s="1">
         <v>45597.512847222199</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>366.03865999999999</v>
@@ -4375,7 +4567,7 @@
         <v>0.14022503226824601</v>
       </c>
       <c r="F8">
-        <v>6.3228362211664404</v>
+        <v>46.983773104811597</v>
       </c>
       <c r="G8">
         <v>68.742208333333295</v>
@@ -4387,29 +4579,30 @@
         <v>3.5498747068957698E-2</v>
       </c>
       <c r="J8">
+        <v>-7.0545003203020098</v>
+      </c>
+      <c r="K8">
         <v>3.4980738563410198E-2</v>
       </c>
-      <c r="K8">
-        <v>1.8441678766639</v>
-      </c>
       <c r="L8">
+        <v>3.8498022890073802</v>
+      </c>
+      <c r="M8">
         <v>-3.3382578769557898</v>
       </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N8">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O8">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A9" s="1">
         <v>45618.559143518498</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <v>2122.394256</v>
@@ -4421,7 +4614,7 @@
         <v>7.67954910734997E-2</v>
       </c>
       <c r="F9">
-        <v>1.04965068409908</v>
+        <v>15.624641446248599</v>
       </c>
       <c r="G9">
         <v>56.827624999999998</v>
@@ -4429,30 +4622,34 @@
       <c r="H9">
         <v>-1.0375902024202499</v>
       </c>
+      <c r="I9">
+        <v>1.3049438876461601</v>
+      </c>
       <c r="J9">
+        <v>-374.777691401879</v>
+      </c>
+      <c r="K9">
         <v>1.0375902024202499</v>
       </c>
-      <c r="K9">
-        <v>4.84574270081604E-2</v>
-      </c>
       <c r="L9">
+        <v>2.7488492479190798</v>
+      </c>
+      <c r="M9">
         <v>0.26616004187793002</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O9">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A10" s="1">
         <v>45639.595601851797</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>335.75364000000002</v>
@@ -4461,29 +4658,27 @@
         <v>5.5228227659252498E-2</v>
       </c>
       <c r="F10">
-        <v>0.39629401292160898</v>
+        <v>8.5709619988180794</v>
       </c>
       <c r="G10">
         <v>51.593166666666697</v>
       </c>
-      <c r="K10">
-        <v>-0.92559888633966103</v>
-      </c>
-      <c r="M10">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
+      <c r="L10">
+        <v>2.1483799782140101</v>
       </c>
       <c r="N10">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O10">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A11" s="1">
         <v>45660.5559027778</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C11">
         <v>335.25396000000001</v>
@@ -4495,7 +4690,7 @@
         <v>5.0095874737204102E-2</v>
       </c>
       <c r="F11">
-        <v>0.295964793657363</v>
+        <v>7.1699172276345804</v>
       </c>
       <c r="G11">
         <v>50.861624999999997</v>
@@ -4507,29 +4702,30 @@
         <v>3.7428936539669E-2</v>
       </c>
       <c r="J11">
+        <v>-14.5652303048023</v>
+      </c>
+      <c r="K11">
         <v>2.6571209433532701E-2</v>
       </c>
-      <c r="K11">
-        <v>-1.21751477207879</v>
-      </c>
       <c r="L11">
+        <v>1.9698941102819301</v>
+      </c>
+      <c r="M11">
         <v>-3.2853111694472799</v>
       </c>
-      <c r="M11">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N11">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O11">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A12" s="1">
         <v>45684.6496527778</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C12">
         <v>365.76996000000003</v>
@@ -4541,7 +4737,7 @@
         <v>0.196666010534818</v>
       </c>
       <c r="F12">
-        <v>17.3515434504375</v>
+        <v>87.224594266290794</v>
       </c>
       <c r="G12">
         <v>50.617791666666697</v>
@@ -4553,29 +4749,30 @@
         <v>0.20618270723144499</v>
       </c>
       <c r="J12">
+        <v>-20.330174292241502</v>
+      </c>
+      <c r="K12">
         <v>0.14566217357103201</v>
       </c>
-      <c r="K12">
-        <v>2.8536814621155799</v>
-      </c>
       <c r="L12">
+        <v>4.4684863354860997</v>
+      </c>
+      <c r="M12">
         <v>-1.57899257497307</v>
       </c>
-      <c r="M12">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N12">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O12">
+        <v>0.47237812690643199</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.75">
       <c r="A13" s="1">
         <v>45742.576273148203</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C13">
         <v>350.31240000000003</v>
@@ -4586,6 +4783,9 @@
       <c r="E13">
         <v>0.109133966298236</v>
       </c>
+      <c r="F13">
+        <v>29.707918352512699</v>
+      </c>
       <c r="G13">
         <v>62.7820416666667</v>
       </c>
@@ -4596,18 +4796,22 @@
         <v>2.2382569309555799E-2</v>
       </c>
       <c r="J13">
+        <v>-5.0977316325946296</v>
+      </c>
+      <c r="K13">
         <v>1.98588897560266E-2</v>
       </c>
       <c r="L13">
+        <v>3.39141362146992</v>
+      </c>
+      <c r="M13">
         <v>-3.7994727788649398</v>
       </c>
-      <c r="M13">
-        <f t="shared" si="0"/>
-        <v>5.6712953735995913E-2</v>
-      </c>
       <c r="N13">
-        <f t="shared" si="1"/>
-        <v>5.8748895691836701E-2</v>
+        <v>0.96253848858725999</v>
+      </c>
+      <c r="O13">
+        <v>0.47237812690643199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>